<commit_message>
Final updates: episode content, host profiles, and links
</commit_message>
<xml_diff>
--- a/Update Web Application.xlsx
+++ b/Update Web Application.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/monikaaggarwal/Documents/2024/Blogs and Posts/Podcast - Agent Sense/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7B6E21A-9EDA-9142-A65F-96EB2924D8B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{208DF983-4474-2840-8261-B9DB91C6E34A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="39200" yWindow="660" windowWidth="32140" windowHeight="19600" xr2:uid="{93B67EED-A597-B54E-8F0F-31385D582193}"/>
   </bookViews>
@@ -123,9 +123,6 @@
 That is the gap between experimentation and production.</t>
   </si>
   <si>
-    <t>n this episode, my co host Frank Chávez and I are joined by Vitalii Duk from Dynamiq to discuss how agents are moving from answering questions to doing work across tools, systems, and runtime environments.. 𝙏𝙝𝙞𝙨 𝙞𝙨 𝙩𝙝𝙚 𝙚𝙣𝙩𝙚𝙧𝙥𝙧𝙞𝙨𝙚 𝙖𝙧𝙘𝙝𝙞𝙩𝙚𝙘𝙩𝙪𝙧𝙚 𝙨𝙝𝙞𝙛𝙩: 𝙖𝙜𝙚𝙣𝙩𝙨 𝙖𝙧𝙚 𝙢𝙤𝙫𝙞𝙣𝙜 𝙛𝙧𝙤𝙢 𝙧𝙚𝙨𝙥𝙤𝙣𝙨𝙚 𝙩𝙤 𝙚𝙭𝙚𝙘𝙪𝙩𝙞𝙤𝙣. 𝙏𝙝𝙚 𝙫𝙖𝙡𝙪𝙚 𝙞𝙨 𝙣𝙤𝙩 𝙤𝙣𝙡𝙮 𝙞𝙣 𝙬𝙝𝙖𝙩 𝙩𝙝𝙚 𝙖𝙜𝙚𝙣𝙩 𝙘𝙖𝙣 𝙙𝙤. 𝙄𝙩 𝙞𝙨 𝙞𝙣 𝙝𝙤𝙬 𝙨𝙖𝙛𝙚𝙡𝙮, 𝙤𝙗𝙨𝙚𝙧𝙫𝙖𝙗𝙡𝙮, 𝙖𝙣𝙙 𝙧𝙚𝙥𝙚𝙖𝙩𝙖𝙗𝙡𝙮 𝙞𝙩 𝙘𝙖𝙣 𝙤𝙥𝙚𝙧𝙖𝙩𝙚 𝙞𝙣 𝙧𝙚𝙖𝙡 𝙗𝙪𝙨𝙞𝙣𝙚𝙨𝙨 𝙬𝙤𝙧𝙠.</t>
-  </si>
-  <si>
     <t>MCP helps agents connect to tools and systems. But connection alone is not enough. As agents start working across ServiceNow, Workday, SAP, HR, IT, finance, and customer operations, enterprises need a control layer.
 That is where the MCP Gateway comes in.
 We discuss how an MCP Gateway helps manage identity, policy, approvals, audit, and traceability. It gives agents access to approved tools without opening direct, unmanaged paths into core enterprise systems.</t>
@@ -149,6 +146,9 @@
   <si>
     <t xml:space="preserve">This episode explores the line between deterministic business logic and autonomous agents in real business operations, using a Commercial and Investment Banking onboarding scenario to show where rules work, where agents help, and where humans must stay in control.
 </t>
+  </si>
+  <si>
+    <t>Guest: Vitalii Duk is the Founder and CEO of Dynamiq. He founded Dynamiq to make agentic AI practical and secure for organizations, simplifying the journey from prototype to production.  We discuss how agents are moving from answering questions to doing work across tools, systems, and runtime environments. 𝙏𝙝𝙞𝙨 𝙞𝙨 𝙩𝙝𝙚 𝙚𝙣𝙩𝙚𝙧𝙥𝙧𝙞𝙨𝙚 𝙖𝙧𝙘𝙝𝙞𝙩𝙚𝙘𝙩𝙪𝙧𝙚 𝙨𝙝𝙞𝙛𝙩: 𝙖𝙜𝙚𝙣𝙩𝙨 𝙖𝙧𝙚 𝙢𝙤𝙫𝙞𝙣𝙜 𝙛𝙧𝙤𝙢 𝙧𝙚𝙨𝙥𝙤𝙣𝙨𝙚 𝙩𝙤 𝙚𝙭𝙚𝙘𝙪𝙩𝙞𝙤𝙣. 𝙏𝙝𝙚 𝙫𝙖𝙡𝙪𝙚 𝙞𝙨 𝙣𝙤𝙩 𝙤𝙣𝙡𝙮 𝙞𝙣 𝙬𝙝𝙖𝙩 𝙩𝙝𝙚 𝙖𝙜𝙚𝙣𝙩 𝙘𝙖𝙣 𝙙𝙤. 𝙄𝙩 𝙞𝙨 𝙞𝙣 𝙝𝙤𝙬 𝙨𝙖𝙛𝙚𝙡𝙮, 𝙤𝙗𝙨𝙚𝙧𝙫𝙖𝙗𝙡𝙮, 𝙖𝙣𝙙 𝙧𝙚𝙥𝙚𝙖𝙩𝙖𝙗𝙡𝙮 𝙞𝙩 𝙘𝙖𝙣 𝙤𝙥𝙚𝙧𝙖𝙩𝙚 𝙞𝙣 𝙧𝙚𝙖𝙡 𝙗𝙪𝙨𝙞𝙣𝙚𝙨𝙨 𝙬𝙤𝙧𝙠.</t>
   </si>
 </sst>
 </file>
@@ -610,7 +610,7 @@
         <v>19</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>5</v>
@@ -628,7 +628,7 @@
         <v>20</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>7</v>
@@ -646,7 +646,7 @@
         <v>21</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>9</v>
@@ -664,7 +664,7 @@
         <v>22</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>11</v>
@@ -682,7 +682,7 @@
         <v>23</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>13</v>
@@ -700,7 +700,7 @@
         <v>24</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>15</v>

</xml_diff>